<commit_message>
idk what is happening here
</commit_message>
<xml_diff>
--- a/Hydroacoustics/TAST/TAST_2025_seal_for_pp_3.xlsx
+++ b/Hydroacoustics/TAST/TAST_2025_seal_for_pp_3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/khadijahhomolka/Documents/GitHub/PGST-Natural-Resources/Hydroacoustics/TAST/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D1768E4C-B4FF-7A4F-AB1E-28C057FCE9D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93F5C0B6-1614-9C41-B468-1A0F30D7CA37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1100" yWindow="820" windowWidth="28040" windowHeight="17440" xr2:uid="{D6D37DE6-2735-C846-9944-0948A4A78BFB}"/>
+    <workbookView xWindow="35700" yWindow="-240" windowWidth="28040" windowHeight="17440" xr2:uid="{D6D37DE6-2735-C846-9944-0948A4A78BFB}"/>
   </bookViews>
   <sheets>
     <sheet name="TAST_2025_seal_for_pp_3" sheetId="1" r:id="rId1"/>
@@ -9015,6 +9015,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55112B20-A5CC-0649-82B3-1A0BF80C172C}">
   <dimension ref="B1:V1344"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="28.33203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B1" t="s">

</xml_diff>